<commit_message>
add llama13b  and embedding code
</commit_message>
<xml_diff>
--- a/llm-mem-exp2.xlsx
+++ b/llm-mem-exp2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/libo15/code/llm-memorization/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C51D1391-4450-424D-95B1-B29F3823820C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74481BA4-760B-5E41-9ACA-A1A862B37E3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="660" yWindow="1000" windowWidth="27840" windowHeight="15440" activeTab="1" xr2:uid="{60BE1878-A98E-2548-9C6F-0ED76844BB32}"/>
+    <workbookView xWindow="660" yWindow="880" windowWidth="27840" windowHeight="15440" xr2:uid="{60BE1878-A98E-2548-9C6F-0ED76844BB32}"/>
   </bookViews>
   <sheets>
     <sheet name="原始数据" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">原始数据!$A$1:$G$271</definedName>
   </definedNames>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -214,7 +214,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -230,16 +230,10 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -4356,7 +4350,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC23FC95-0A9A-3140-A7F3-93D8E7B6A2F6}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:G271"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
@@ -4668,7 +4661,7 @@
         <v>3.1450921289970601</v>
       </c>
     </row>
-    <row r="14" spans="1:7" hidden="1">
+    <row r="14" spans="1:7">
       <c r="A14" s="2">
         <v>13</v>
       </c>
@@ -4714,7 +4707,7 @@
         <v>1.84683167549835</v>
       </c>
     </row>
-    <row r="16" spans="1:7" hidden="1">
+    <row r="16" spans="1:7">
       <c r="A16" s="2">
         <v>15</v>
       </c>
@@ -4737,7 +4730,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:7" hidden="1">
+    <row r="17" spans="1:7">
       <c r="A17" s="2">
         <v>16</v>
       </c>
@@ -4760,7 +4753,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:7" hidden="1">
+    <row r="18" spans="1:7">
       <c r="A18" s="2">
         <v>17</v>
       </c>
@@ -4806,7 +4799,7 @@
         <v>2.5806821886629199</v>
       </c>
     </row>
-    <row r="20" spans="1:7" hidden="1">
+    <row r="20" spans="1:7">
       <c r="A20" s="2">
         <v>19</v>
       </c>
@@ -4967,7 +4960,7 @@
         <v>2.8219079803913201</v>
       </c>
     </row>
-    <row r="27" spans="1:7" hidden="1">
+    <row r="27" spans="1:7">
       <c r="A27" s="2">
         <v>26</v>
       </c>
@@ -5036,7 +5029,7 @@
         <v>2.9616866315173902</v>
       </c>
     </row>
-    <row r="30" spans="1:7" hidden="1">
+    <row r="30" spans="1:7">
       <c r="A30" s="2">
         <v>29</v>
       </c>
@@ -5266,7 +5259,7 @@
         <v>2.3990793434618398</v>
       </c>
     </row>
-    <row r="40" spans="1:7" hidden="1">
+    <row r="40" spans="1:7">
       <c r="A40" s="2">
         <v>39</v>
       </c>
@@ -5358,7 +5351,7 @@
         <v>3.0776937232589399</v>
       </c>
     </row>
-    <row r="44" spans="1:7" hidden="1">
+    <row r="44" spans="1:7">
       <c r="A44" s="2">
         <v>43</v>
       </c>
@@ -5381,7 +5374,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:7" hidden="1">
+    <row r="45" spans="1:7">
       <c r="A45" s="2">
         <v>44</v>
       </c>
@@ -5519,7 +5512,7 @@
         <v>2.6104098983278101</v>
       </c>
     </row>
-    <row r="51" spans="1:7" hidden="1">
+    <row r="51" spans="1:7">
       <c r="A51" s="2">
         <v>50</v>
       </c>
@@ -5611,7 +5604,7 @@
         <v>3.0301913973071302</v>
       </c>
     </row>
-    <row r="55" spans="1:7" hidden="1">
+    <row r="55" spans="1:7">
       <c r="A55" s="2">
         <v>54</v>
       </c>
@@ -5634,7 +5627,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:7" hidden="1">
+    <row r="56" spans="1:7">
       <c r="A56" s="2">
         <v>55</v>
       </c>
@@ -5726,7 +5719,7 @@
         <v>3.18163790221283</v>
       </c>
     </row>
-    <row r="60" spans="1:7" hidden="1">
+    <row r="60" spans="1:7">
       <c r="A60" s="2">
         <v>59</v>
       </c>
@@ -6002,7 +5995,7 @@
         <v>2.8422128301349301</v>
       </c>
     </row>
-    <row r="72" spans="1:7" hidden="1">
+    <row r="72" spans="1:7">
       <c r="A72" s="2">
         <v>71</v>
       </c>
@@ -6255,7 +6248,7 @@
         <v>3.1933337633269501</v>
       </c>
     </row>
-    <row r="83" spans="1:7" hidden="1">
+    <row r="83" spans="1:7">
       <c r="A83" s="2">
         <v>82</v>
       </c>
@@ -6301,7 +6294,7 @@
         <v>3.1978976367216299</v>
       </c>
     </row>
-    <row r="85" spans="1:7" hidden="1">
+    <row r="85" spans="1:7">
       <c r="A85" s="2">
         <v>84</v>
       </c>
@@ -6393,7 +6386,7 @@
         <v>2.9053917055926699</v>
       </c>
     </row>
-    <row r="89" spans="1:7" hidden="1">
+    <row r="89" spans="1:7">
       <c r="A89" s="2">
         <v>88</v>
       </c>
@@ -6439,7 +6432,7 @@
         <v>2.93284339999905</v>
       </c>
     </row>
-    <row r="91" spans="1:7" hidden="1">
+    <row r="91" spans="1:7">
       <c r="A91" s="2">
         <v>90</v>
       </c>
@@ -6485,7 +6478,7 @@
         <v>3.1763192931908399</v>
       </c>
     </row>
-    <row r="93" spans="1:7" hidden="1">
+    <row r="93" spans="1:7">
       <c r="A93" s="2">
         <v>92</v>
       </c>
@@ -6577,7 +6570,7 @@
         <v>3.2868986291993001</v>
       </c>
     </row>
-    <row r="97" spans="1:7" hidden="1">
+    <row r="97" spans="1:7">
       <c r="A97" s="2">
         <v>96</v>
       </c>
@@ -6600,7 +6593,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="98" spans="1:7" hidden="1">
+    <row r="98" spans="1:7">
       <c r="A98" s="2">
         <v>97</v>
       </c>
@@ -6784,7 +6777,7 @@
         <v>3.2635859131590399</v>
       </c>
     </row>
-    <row r="106" spans="1:7" hidden="1">
+    <row r="106" spans="1:7">
       <c r="A106" s="2">
         <v>105</v>
       </c>
@@ -6876,7 +6869,7 @@
         <v>3.1853567622433201</v>
       </c>
     </row>
-    <row r="110" spans="1:7" hidden="1">
+    <row r="110" spans="1:7">
       <c r="A110" s="2">
         <v>109</v>
       </c>
@@ -6968,7 +6961,7 @@
         <v>3.1365747363838499</v>
       </c>
     </row>
-    <row r="114" spans="1:7" hidden="1">
+    <row r="114" spans="1:7">
       <c r="A114" s="2">
         <v>113</v>
       </c>
@@ -7014,7 +7007,7 @@
         <v>3.0451022072758498</v>
       </c>
     </row>
-    <row r="116" spans="1:7" hidden="1">
+    <row r="116" spans="1:7">
       <c r="A116" s="2">
         <v>115</v>
       </c>
@@ -7037,7 +7030,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="1:7" hidden="1">
+    <row r="117" spans="1:7">
       <c r="A117" s="2">
         <v>116</v>
       </c>
@@ -7060,7 +7053,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="1:7" hidden="1">
+    <row r="118" spans="1:7">
       <c r="A118" s="2">
         <v>117</v>
       </c>
@@ -7175,7 +7168,7 @@
         <v>2.6490086393253498</v>
       </c>
     </row>
-    <row r="123" spans="1:7" hidden="1">
+    <row r="123" spans="1:7">
       <c r="A123" s="2">
         <v>122</v>
       </c>
@@ -7244,7 +7237,7 @@
         <v>3.2247010886707201</v>
       </c>
     </row>
-    <row r="126" spans="1:7" hidden="1">
+    <row r="126" spans="1:7">
       <c r="A126" s="2">
         <v>125</v>
       </c>
@@ -7290,7 +7283,7 @@
         <v>1.82626332828088</v>
       </c>
     </row>
-    <row r="128" spans="1:7" hidden="1">
+    <row r="128" spans="1:7">
       <c r="A128" s="2">
         <v>127</v>
       </c>
@@ -7520,7 +7513,7 @@
         <v>3.1441624554410299</v>
       </c>
     </row>
-    <row r="138" spans="1:7" hidden="1">
+    <row r="138" spans="1:7">
       <c r="A138" s="2">
         <v>137</v>
       </c>
@@ -7612,7 +7605,7 @@
         <v>3.0916275931058999</v>
       </c>
     </row>
-    <row r="142" spans="1:7" hidden="1">
+    <row r="142" spans="1:7">
       <c r="A142" s="2">
         <v>141</v>
       </c>
@@ -7704,7 +7697,7 @@
         <v>2.8150083691651799</v>
       </c>
     </row>
-    <row r="146" spans="1:7" hidden="1">
+    <row r="146" spans="1:7">
       <c r="A146" s="2">
         <v>145</v>
       </c>
@@ -7750,7 +7743,7 @@
         <v>2.8140503352635502</v>
       </c>
     </row>
-    <row r="148" spans="1:7" hidden="1">
+    <row r="148" spans="1:7">
       <c r="A148" s="2">
         <v>147</v>
       </c>
@@ -7865,7 +7858,7 @@
         <v>2.7397141791042698</v>
       </c>
     </row>
-    <row r="153" spans="1:7" hidden="1">
+    <row r="153" spans="1:7">
       <c r="A153" s="2">
         <v>152</v>
       </c>
@@ -7888,7 +7881,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="154" spans="1:7" hidden="1">
+    <row r="154" spans="1:7">
       <c r="A154" s="2">
         <v>153</v>
       </c>
@@ -7980,7 +7973,7 @@
         <v>2.6857838834038401</v>
       </c>
     </row>
-    <row r="158" spans="1:7" hidden="1">
+    <row r="158" spans="1:7">
       <c r="A158" s="2">
         <v>157</v>
       </c>
@@ -8210,7 +8203,7 @@
         <v>3.1330635939410501</v>
       </c>
     </row>
-    <row r="168" spans="1:7" hidden="1">
+    <row r="168" spans="1:7">
       <c r="A168" s="2">
         <v>167</v>
       </c>
@@ -8256,7 +8249,7 @@
         <v>3.2509225855491199</v>
       </c>
     </row>
-    <row r="170" spans="1:7" hidden="1">
+    <row r="170" spans="1:7">
       <c r="A170" s="2">
         <v>169</v>
       </c>
@@ -8417,7 +8410,7 @@
         <v>2.9703745886642698</v>
       </c>
     </row>
-    <row r="177" spans="1:7" hidden="1">
+    <row r="177" spans="1:7">
       <c r="A177" s="2">
         <v>176</v>
       </c>
@@ -8440,7 +8433,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="178" spans="1:7" hidden="1">
+    <row r="178" spans="1:7">
       <c r="A178" s="2">
         <v>177</v>
       </c>
@@ -8509,7 +8502,7 @@
         <v>3.1869961765599699</v>
       </c>
     </row>
-    <row r="181" spans="1:7" hidden="1">
+    <row r="181" spans="1:7">
       <c r="A181" s="2">
         <v>180</v>
       </c>
@@ -8601,7 +8594,7 @@
         <v>2.9766185183685399</v>
       </c>
     </row>
-    <row r="185" spans="1:7" hidden="1">
+    <row r="185" spans="1:7">
       <c r="A185" s="2">
         <v>184</v>
       </c>
@@ -8716,7 +8709,7 @@
         <v>3.07608691609239</v>
       </c>
     </row>
-    <row r="190" spans="1:7" hidden="1">
+    <row r="190" spans="1:7">
       <c r="A190" s="2">
         <v>189</v>
       </c>
@@ -8785,7 +8778,7 @@
         <v>2.9252338181994002</v>
       </c>
     </row>
-    <row r="193" spans="1:7" hidden="1">
+    <row r="193" spans="1:7">
       <c r="A193" s="2">
         <v>192</v>
       </c>
@@ -8808,7 +8801,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="194" spans="1:7" hidden="1">
+    <row r="194" spans="1:7">
       <c r="A194" s="2">
         <v>193</v>
       </c>
@@ -8854,7 +8847,7 @@
         <v>2.71101412295921</v>
       </c>
     </row>
-    <row r="196" spans="1:7" hidden="1">
+    <row r="196" spans="1:7">
       <c r="A196" s="2">
         <v>195</v>
       </c>
@@ -8900,7 +8893,7 @@
         <v>2.9600513572635299</v>
       </c>
     </row>
-    <row r="198" spans="1:7" hidden="1">
+    <row r="198" spans="1:7">
       <c r="A198" s="2">
         <v>197</v>
       </c>
@@ -8946,7 +8939,7 @@
         <v>2.4257325481805898</v>
       </c>
     </row>
-    <row r="200" spans="1:7" hidden="1">
+    <row r="200" spans="1:7">
       <c r="A200" s="2">
         <v>199</v>
       </c>
@@ -9199,7 +9192,7 @@
         <v>2.8368103404474101</v>
       </c>
     </row>
-    <row r="211" spans="1:7" hidden="1">
+    <row r="211" spans="1:7">
       <c r="A211" s="2">
         <v>210</v>
       </c>
@@ -9383,7 +9376,7 @@
         <v>3.26773584411024</v>
       </c>
     </row>
-    <row r="219" spans="1:7" hidden="1">
+    <row r="219" spans="1:7">
       <c r="A219" s="2">
         <v>218</v>
       </c>
@@ -9406,7 +9399,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="220" spans="1:7" hidden="1">
+    <row r="220" spans="1:7">
       <c r="A220" s="2">
         <v>219</v>
       </c>
@@ -9544,7 +9537,7 @@
         <v>2.8391126188994602</v>
       </c>
     </row>
-    <row r="226" spans="1:7" hidden="1">
+    <row r="226" spans="1:7">
       <c r="A226" s="2">
         <v>225</v>
       </c>
@@ -9659,7 +9652,7 @@
         <v>3.2003549114354</v>
       </c>
     </row>
-    <row r="231" spans="1:7" hidden="1">
+    <row r="231" spans="1:7">
       <c r="A231" s="2">
         <v>230</v>
       </c>
@@ -9728,7 +9721,7 @@
         <v>3.1968680305664399</v>
       </c>
     </row>
-    <row r="234" spans="1:7" hidden="1">
+    <row r="234" spans="1:7">
       <c r="A234" s="2">
         <v>233</v>
       </c>
@@ -9843,7 +9836,7 @@
         <v>3.1698163972852602</v>
       </c>
     </row>
-    <row r="239" spans="1:7" hidden="1">
+    <row r="239" spans="1:7">
       <c r="A239" s="2">
         <v>238</v>
       </c>
@@ -10050,7 +10043,7 @@
         <v>3.2451173944264902</v>
       </c>
     </row>
-    <row r="248" spans="1:7" hidden="1">
+    <row r="248" spans="1:7">
       <c r="A248" s="2">
         <v>247</v>
       </c>
@@ -10119,7 +10112,7 @@
         <v>3.1427014932402599</v>
       </c>
     </row>
-    <row r="251" spans="1:7" hidden="1">
+    <row r="251" spans="1:7">
       <c r="A251" s="2">
         <v>250</v>
       </c>
@@ -10211,7 +10204,7 @@
         <v>3.06309455909309</v>
       </c>
     </row>
-    <row r="255" spans="1:7" hidden="1">
+    <row r="255" spans="1:7">
       <c r="A255" s="2">
         <v>254</v>
       </c>
@@ -10326,7 +10319,7 @@
         <v>2.91978859687512</v>
       </c>
     </row>
-    <row r="260" spans="1:7" hidden="1">
+    <row r="260" spans="1:7">
       <c r="A260" s="2">
         <v>259</v>
       </c>
@@ -10418,7 +10411,7 @@
         <v>1.99700566556244</v>
       </c>
     </row>
-    <row r="264" spans="1:7" hidden="1">
+    <row r="264" spans="1:7">
       <c r="A264" s="2">
         <v>263</v>
       </c>
@@ -10487,7 +10480,7 @@
         <v>3.2812053853033798</v>
       </c>
     </row>
-    <row r="267" spans="1:7" hidden="1">
+    <row r="267" spans="1:7">
       <c r="A267" s="2">
         <v>266</v>
       </c>
@@ -10533,7 +10526,7 @@
         <v>1.9451348598007501</v>
       </c>
     </row>
-    <row r="269" spans="1:7" hidden="1">
+    <row r="269" spans="1:7">
       <c r="A269" s="2">
         <v>268</v>
       </c>
@@ -10603,213 +10596,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G271" xr:uid="{EC23FC95-0A9A-3140-A7F3-93D8E7B6A2F6}">
-    <filterColumn colId="4">
-      <filters>
-        <filter val="0.049650852"/>
-        <filter val="0.053677995"/>
-        <filter val="0.055080205"/>
-        <filter val="0.058746267"/>
-        <filter val="0.060963564"/>
-        <filter val="0.061959922"/>
-        <filter val="0.062901199"/>
-        <filter val="0.062956199"/>
-        <filter val="0.06565699"/>
-        <filter val="0.066406488"/>
-        <filter val="0.068241544"/>
-        <filter val="0.071240209"/>
-        <filter val="0.073560886"/>
-        <filter val="0.076544695"/>
-        <filter val="0.077858403"/>
-        <filter val="0.080336317"/>
-        <filter val="0.085432656"/>
-        <filter val="0.088209867"/>
-        <filter val="0.088940024"/>
-        <filter val="0.089927174"/>
-        <filter val="0.096570276"/>
-        <filter val="0.097323999"/>
-        <filter val="0.108440027"/>
-        <filter val="0.128569588"/>
-        <filter val="0.135189716"/>
-        <filter val="0.140937582"/>
-        <filter val="0.160325751"/>
-        <filter val="0.164996061"/>
-        <filter val="0.16529892"/>
-        <filter val="0.167777613"/>
-        <filter val="0.171568662"/>
-        <filter val="0.175893335"/>
-        <filter val="0.176691622"/>
-        <filter val="0.179115757"/>
-        <filter val="0.185535029"/>
-        <filter val="0.198900163"/>
-        <filter val="0.205551331"/>
-        <filter val="0.20888488"/>
-        <filter val="0.218915366"/>
-        <filter val="0.232767399"/>
-        <filter val="0.240045667"/>
-        <filter val="0.25114977"/>
-        <filter val="0.256025121"/>
-        <filter val="0.260228243"/>
-        <filter val="0.263965754"/>
-        <filter val="0.266304846"/>
-        <filter val="0.271527608"/>
-        <filter val="0.279232927"/>
-        <filter val="0.287163734"/>
-        <filter val="0.290525258"/>
-        <filter val="0.297915027"/>
-        <filter val="0.302718945"/>
-        <filter val="0.304329604"/>
-        <filter val="0.314400725"/>
-        <filter val="0.319628267"/>
-        <filter val="0.319993304"/>
-        <filter val="0.330003694"/>
-        <filter val="0.33105775"/>
-        <filter val="0.351762604"/>
-        <filter val="0.352621814"/>
-        <filter val="0.363225326"/>
-        <filter val="0.367313698"/>
-        <filter val="0.369216383"/>
-        <filter val="0.381974712"/>
-        <filter val="0.393325686"/>
-        <filter val="0.395924829"/>
-        <filter val="0.401465872"/>
-        <filter val="0.405920684"/>
-        <filter val="0.407837987"/>
-        <filter val="0.415520955"/>
-        <filter val="0.416180318"/>
-        <filter val="0.41654776"/>
-        <filter val="0.418802986"/>
-        <filter val="0.42128139"/>
-        <filter val="0.423429053"/>
-        <filter val="0.423922643"/>
-        <filter val="0.424922962"/>
-        <filter val="0.425480748"/>
-        <filter val="0.434540665"/>
-        <filter val="0.436009724"/>
-        <filter val="0.436857544"/>
-        <filter val="0.442534698"/>
-        <filter val="0.449147007"/>
-        <filter val="0.463598981"/>
-        <filter val="0.465614077"/>
-        <filter val="0.466169316"/>
-        <filter val="0.470719192"/>
-        <filter val="0.479424994"/>
-        <filter val="0.481252877"/>
-        <filter val="0.482420415"/>
-        <filter val="0.482662755"/>
-        <filter val="0.489336263"/>
-        <filter val="0.490070254"/>
-        <filter val="0.490365793"/>
-        <filter val="0.491944885"/>
-        <filter val="0.492331937"/>
-        <filter val="0.493467333"/>
-        <filter val="0.493643317"/>
-        <filter val="0.498253547"/>
-        <filter val="0.499400099"/>
-        <filter val="0.503076342"/>
-        <filter val="0.503108611"/>
-        <filter val="0.506809273"/>
-        <filter val="0.507718779"/>
-        <filter val="0.508237774"/>
-        <filter val="0.511016756"/>
-        <filter val="0.512244264"/>
-        <filter val="0.513703456"/>
-        <filter val="0.513808455"/>
-        <filter val="0.514199726"/>
-        <filter val="0.516959447"/>
-        <filter val="0.517154551"/>
-        <filter val="0.51862675"/>
-        <filter val="0.519324465"/>
-        <filter val="0.519875514"/>
-        <filter val="0.520607149"/>
-        <filter val="0.522000417"/>
-        <filter val="0.522027198"/>
-        <filter val="0.524145104"/>
-        <filter val="0.524255335"/>
-        <filter val="0.52607435"/>
-        <filter val="0.53255827"/>
-        <filter val="0.537093242"/>
-        <filter val="0.540812995"/>
-        <filter val="0.543840257"/>
-        <filter val="0.544670518"/>
-        <filter val="0.548633317"/>
-        <filter val="0.54943375"/>
-        <filter val="0.551242948"/>
-        <filter val="0.557285951"/>
-        <filter val="0.564414054"/>
-        <filter val="0.566042647"/>
-        <filter val="0.572689004"/>
-        <filter val="0.572836156"/>
-        <filter val="0.57411959"/>
-        <filter val="0.583996318"/>
-        <filter val="0.589712226"/>
-        <filter val="0.592183486"/>
-        <filter val="0.592885505"/>
-        <filter val="0.593103233"/>
-        <filter val="0.593173523"/>
-        <filter val="0.593749054"/>
-        <filter val="0.594213275"/>
-        <filter val="0.594618876"/>
-        <filter val="0.595212743"/>
-        <filter val="0.595437061"/>
-        <filter val="0.597178534"/>
-        <filter val="0.604902342"/>
-        <filter val="0.606237337"/>
-        <filter val="0.609610587"/>
-        <filter val="0.610517859"/>
-        <filter val="0.612944644"/>
-        <filter val="0.614111871"/>
-        <filter val="0.614727508"/>
-        <filter val="0.61771984"/>
-        <filter val="0.619046507"/>
-        <filter val="0.619072547"/>
-        <filter val="0.619676698"/>
-        <filter val="0.620127797"/>
-        <filter val="0.625643045"/>
-        <filter val="0.632013813"/>
-        <filter val="0.644021571"/>
-        <filter val="0.648509653"/>
-        <filter val="0.64962665"/>
-        <filter val="0.654749796"/>
-        <filter val="0.663724508"/>
-        <filter val="0.670115739"/>
-        <filter val="0.671433747"/>
-        <filter val="0.673971534"/>
-        <filter val="0.676940322"/>
-        <filter val="0.682890415"/>
-        <filter val="0.684101656"/>
-        <filter val="0.68857265"/>
-        <filter val="0.689903575"/>
-        <filter val="0.691644229"/>
-        <filter val="0.69240348"/>
-        <filter val="0.694065134"/>
-        <filter val="0.701858872"/>
-        <filter val="0.703650375"/>
-        <filter val="0.707752446"/>
-        <filter val="0.709090811"/>
-        <filter val="0.72904405"/>
-        <filter val="0.730640481"/>
-        <filter val="0.732212186"/>
-        <filter val="0.732241078"/>
-        <filter val="0.767191112"/>
-        <filter val="0.775148645"/>
-        <filter val="0.780234343"/>
-        <filter val="0.781746924"/>
-        <filter val="0.785906708"/>
-        <filter val="0.798038423"/>
-        <filter val="0.812963471"/>
-        <filter val="0.821524501"/>
-        <filter val="0.835539925"/>
-        <filter val="0.83850652"/>
-        <filter val="0.853841643"/>
-        <filter val="0.857771114"/>
-        <filter val="0.858622571"/>
-        <filter val="0.909231683"/>
-        <filter val="0.922650051"/>
-        <filter val="0.963334739"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:G271" xr:uid="{EC23FC95-0A9A-3140-A7F3-93D8E7B6A2F6}"/>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -10820,7 +10607,7 @@
   <dimension ref="A1:AL207"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
-    <col min="1" max="1" width="3.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.33203125" customWidth="1"/>
     <col min="2" max="2" width="20.5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="22" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="24.5" bestFit="1" customWidth="1"/>
@@ -12746,40 +12533,40 @@
       <c r="G43" s="2">
         <v>3.0301913973071302</v>
       </c>
-      <c r="K43" s="8" t="s">
+      <c r="K43" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="L43" s="8" t="s">
+      <c r="L43" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="N43" s="8" t="s">
+      <c r="N43" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="O43" s="8" t="s">
+      <c r="O43" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="T43" s="8" t="s">
+      <c r="T43" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="U43" s="8" t="s">
+      <c r="U43" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="W43" s="8" t="s">
+      <c r="W43" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="X43" s="8" t="s">
+      <c r="X43" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="AC43" s="8" t="s">
+      <c r="AC43" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="AD43" s="8" t="s">
+      <c r="AD43" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="AF43" s="8" t="s">
+      <c r="AF43" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="AG43" s="8" t="s">
+      <c r="AG43" s="6" t="s">
         <v>16</v>
       </c>
     </row>
@@ -12805,63 +12592,63 @@
       <c r="G44" s="2">
         <v>3.3024639185577001</v>
       </c>
-      <c r="K44" s="10">
+      <c r="K44" s="8">
         <v>0.21419134736060999</v>
       </c>
-      <c r="L44" s="6">
+      <c r="L44">
         <v>1</v>
       </c>
-      <c r="M44" s="12">
+      <c r="M44" s="10">
         <f>L44/L$65</f>
         <v>4.8543689320388345E-3</v>
       </c>
-      <c r="N44" s="10">
+      <c r="N44" s="8">
         <v>4.9650851637125001E-2</v>
       </c>
-      <c r="O44" s="6">
+      <c r="O44">
         <v>1</v>
       </c>
-      <c r="P44" s="12">
+      <c r="P44" s="10">
         <f>O44/O$65</f>
         <v>4.8543689320388345E-3</v>
       </c>
-      <c r="T44" s="5">
+      <c r="T44" s="1">
         <v>-3.33332680504465E-2</v>
       </c>
-      <c r="U44" s="6">
+      <c r="U44">
         <v>1</v>
       </c>
-      <c r="V44" s="12">
+      <c r="V44" s="10">
         <f>U44/U$65</f>
         <v>4.8543689320388345E-3</v>
       </c>
-      <c r="W44" s="5">
+      <c r="W44" s="1">
         <v>-2.7250470156036301E-2</v>
       </c>
-      <c r="X44" s="6">
+      <c r="X44">
         <v>1</v>
       </c>
-      <c r="Y44" s="12">
+      <c r="Y44" s="10">
         <f>X44/X$65</f>
         <v>4.8780487804878049E-3</v>
       </c>
-      <c r="AC44" s="5">
+      <c r="AC44" s="1">
         <v>2.4611392495922502</v>
       </c>
-      <c r="AD44" s="6">
+      <c r="AD44">
         <v>1</v>
       </c>
-      <c r="AE44" s="12">
+      <c r="AE44" s="10">
         <f>AD44/AD$65</f>
         <v>4.8780487804878049E-3</v>
       </c>
-      <c r="AF44" s="5">
+      <c r="AF44" s="1">
         <v>1.7975936863047199</v>
       </c>
-      <c r="AG44" s="6">
+      <c r="AG44">
         <v>1</v>
       </c>
-      <c r="AH44" s="12">
+      <c r="AH44" s="10">
         <f>AG44/AG$65</f>
         <v>4.8543689320388345E-3</v>
       </c>
@@ -12888,63 +12675,63 @@
       <c r="G45" s="2">
         <v>2.7381257903402401</v>
       </c>
-      <c r="K45" s="10">
+      <c r="K45" s="8">
         <v>0.25390974314589154</v>
       </c>
-      <c r="L45" s="6">
+      <c r="L45">
         <v>1</v>
       </c>
-      <c r="M45" s="12">
+      <c r="M45" s="10">
         <f t="shared" ref="M45:M63" si="9">L45/L$65</f>
         <v>4.8543689320388345E-3</v>
       </c>
-      <c r="N45" s="10">
+      <c r="N45" s="8">
         <v>9.7739477298761632E-2</v>
       </c>
-      <c r="O45" s="6">
+      <c r="O45">
         <v>21</v>
       </c>
-      <c r="P45" s="12">
+      <c r="P45" s="10">
         <f t="shared" ref="P45:P63" si="10">O45/O$65</f>
         <v>0.10194174757281553</v>
       </c>
-      <c r="T45" s="5">
+      <c r="T45" s="1">
         <v>-2.8805170480149432E-2</v>
       </c>
-      <c r="U45" s="6">
+      <c r="U45">
         <v>2</v>
       </c>
-      <c r="V45" s="12">
+      <c r="V45" s="10">
         <f t="shared" ref="V45:V63" si="11">U45/U$65</f>
         <v>9.7087378640776691E-3</v>
       </c>
-      <c r="W45" s="5">
+      <c r="W45" s="1">
         <v>-2.2599660999258555E-2</v>
       </c>
-      <c r="X45" s="6">
-        <v>0</v>
-      </c>
-      <c r="Y45" s="12">
+      <c r="X45">
+        <v>0</v>
+      </c>
+      <c r="Y45" s="10">
         <f t="shared" ref="Y45:Y63" si="12">X45/X$65</f>
         <v>0</v>
       </c>
-      <c r="AC45" s="5">
+      <c r="AC45" s="1">
         <v>2.5126133016959296</v>
       </c>
-      <c r="AD45" s="6">
+      <c r="AD45">
         <v>1</v>
       </c>
-      <c r="AE45" s="12">
+      <c r="AE45" s="10">
         <f t="shared" ref="AE45:AE63" si="13">AD45/AD$65</f>
         <v>4.8780487804878049E-3</v>
       </c>
-      <c r="AF45" s="5">
+      <c r="AF45" s="1">
         <v>1.8935209199908778</v>
       </c>
-      <c r="AG45" s="6">
+      <c r="AG45">
         <v>10</v>
       </c>
-      <c r="AH45" s="12">
+      <c r="AH45" s="10">
         <f t="shared" ref="AH45:AH63" si="14">AG45/AG$65</f>
         <v>4.8543689320388349E-2</v>
       </c>
@@ -12971,63 +12758,63 @@
       <c r="G46" s="2">
         <v>3.18163790221283</v>
       </c>
-      <c r="K46" s="10">
+      <c r="K46" s="8">
         <v>0.29362813893117312</v>
       </c>
-      <c r="L46" s="6">
+      <c r="L46">
         <v>1</v>
       </c>
-      <c r="M46" s="12">
+      <c r="M46" s="10">
         <f t="shared" si="9"/>
         <v>4.8543689320388345E-3</v>
       </c>
-      <c r="N46" s="10">
+      <c r="N46" s="8">
         <v>0.14582810296039828</v>
       </c>
-      <c r="O46" s="6">
+      <c r="O46">
         <v>4</v>
       </c>
-      <c r="P46" s="12">
+      <c r="P46" s="10">
         <f t="shared" si="10"/>
         <v>1.9417475728155338E-2</v>
       </c>
-      <c r="T46" s="5">
+      <c r="T46" s="1">
         <v>-2.4277072909852364E-2</v>
       </c>
-      <c r="U46" s="6">
+      <c r="U46">
         <v>1</v>
       </c>
-      <c r="V46" s="12">
+      <c r="V46" s="10">
         <f t="shared" si="11"/>
         <v>4.8543689320388345E-3</v>
       </c>
-      <c r="W46" s="5">
+      <c r="W46" s="1">
         <v>-1.7948851842480809E-2</v>
       </c>
-      <c r="X46" s="6">
+      <c r="X46">
         <v>4</v>
       </c>
-      <c r="Y46" s="12">
+      <c r="Y46" s="10">
         <f t="shared" si="12"/>
         <v>1.9512195121951219E-2</v>
       </c>
-      <c r="AC46" s="5">
+      <c r="AC46" s="1">
         <v>2.5640873537996089</v>
       </c>
-      <c r="AD46" s="6">
-        <v>0</v>
-      </c>
-      <c r="AE46" s="12">
+      <c r="AD46">
+        <v>0</v>
+      </c>
+      <c r="AE46" s="10">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="AF46" s="5">
+      <c r="AF46" s="1">
         <v>1.9894481536770356</v>
       </c>
-      <c r="AG46" s="6">
+      <c r="AG46">
         <v>5</v>
       </c>
-      <c r="AH46" s="12">
+      <c r="AH46" s="10">
         <f t="shared" si="14"/>
         <v>2.4271844660194174E-2</v>
       </c>
@@ -13054,63 +12841,63 @@
       <c r="G47" s="2">
         <v>3.0544730157062001</v>
       </c>
-      <c r="K47" s="10">
+      <c r="K47" s="8">
         <v>0.3333465347164547</v>
       </c>
-      <c r="L47" s="6">
+      <c r="L47">
         <v>1</v>
       </c>
-      <c r="M47" s="12">
+      <c r="M47" s="10">
         <f t="shared" si="9"/>
         <v>4.8543689320388345E-3</v>
       </c>
-      <c r="N47" s="10">
+      <c r="N47" s="8">
         <v>0.19391672862203491</v>
       </c>
-      <c r="O47" s="6">
+      <c r="O47">
         <v>10</v>
       </c>
-      <c r="P47" s="12">
+      <c r="P47" s="10">
         <f t="shared" si="10"/>
         <v>4.8543689320388349E-2</v>
       </c>
-      <c r="T47" s="5">
+      <c r="T47" s="1">
         <v>-1.9748975339555296E-2</v>
       </c>
-      <c r="U47" s="6">
+      <c r="U47">
         <v>2</v>
       </c>
-      <c r="V47" s="12">
+      <c r="V47" s="10">
         <f t="shared" si="11"/>
         <v>9.7087378640776691E-3</v>
       </c>
-      <c r="W47" s="5">
+      <c r="W47" s="1">
         <v>-1.3298042685703063E-2</v>
       </c>
-      <c r="X47" s="6">
+      <c r="X47">
         <v>10</v>
       </c>
-      <c r="Y47" s="12">
+      <c r="Y47" s="10">
         <f t="shared" si="12"/>
         <v>4.878048780487805E-2</v>
       </c>
-      <c r="AC47" s="5">
+      <c r="AC47" s="1">
         <v>2.6155614059032883</v>
       </c>
-      <c r="AD47" s="6">
-        <v>0</v>
-      </c>
-      <c r="AE47" s="12">
+      <c r="AD47">
+        <v>0</v>
+      </c>
+      <c r="AE47" s="10">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="AF47" s="5">
+      <c r="AF47" s="1">
         <v>2.0853753873631935</v>
       </c>
-      <c r="AG47" s="6">
+      <c r="AG47">
         <v>4</v>
       </c>
-      <c r="AH47" s="12">
+      <c r="AH47" s="10">
         <f t="shared" si="14"/>
         <v>1.9417475728155338E-2</v>
       </c>
@@ -13137,63 +12924,63 @@
       <c r="G48" s="2">
         <v>3.2403517185136499</v>
       </c>
-      <c r="K48" s="10">
+      <c r="K48" s="8">
         <v>0.37306493050173628</v>
       </c>
-      <c r="L48" s="6">
-        <v>0</v>
-      </c>
-      <c r="M48" s="12">
+      <c r="L48">
+        <v>0</v>
+      </c>
+      <c r="M48" s="10">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="N48" s="10">
+      <c r="N48" s="8">
         <v>0.24200535428367154</v>
       </c>
-      <c r="O48" s="6">
+      <c r="O48">
         <v>6</v>
       </c>
-      <c r="P48" s="12">
+      <c r="P48" s="10">
         <f t="shared" si="10"/>
         <v>2.9126213592233011E-2</v>
       </c>
-      <c r="T48" s="5">
+      <c r="T48" s="1">
         <v>-1.5220877769258227E-2</v>
       </c>
-      <c r="U48" s="6">
+      <c r="U48">
         <v>4</v>
       </c>
-      <c r="V48" s="12">
+      <c r="V48" s="10">
         <f t="shared" si="11"/>
         <v>1.9417475728155338E-2</v>
       </c>
-      <c r="W48" s="5">
+      <c r="W48" s="1">
         <v>-8.6472335289253174E-3</v>
       </c>
-      <c r="X48" s="6">
+      <c r="X48">
         <v>7</v>
       </c>
-      <c r="Y48" s="12">
+      <c r="Y48" s="10">
         <f t="shared" si="12"/>
         <v>3.4146341463414637E-2</v>
       </c>
-      <c r="AC48" s="5">
+      <c r="AC48" s="1">
         <v>2.6670354580069677</v>
       </c>
-      <c r="AD48" s="6">
-        <v>0</v>
-      </c>
-      <c r="AE48" s="12">
+      <c r="AD48">
+        <v>0</v>
+      </c>
+      <c r="AE48" s="10">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="AF48" s="5">
+      <c r="AF48" s="1">
         <v>2.1813026210493516</v>
       </c>
-      <c r="AG48" s="6">
-        <v>0</v>
-      </c>
-      <c r="AH48" s="12">
+      <c r="AG48">
+        <v>0</v>
+      </c>
+      <c r="AH48" s="10">
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
@@ -13220,63 +13007,63 @@
       <c r="G49" s="2">
         <v>3.1418011168453699</v>
       </c>
-      <c r="K49" s="10">
+      <c r="K49" s="8">
         <v>0.41278332628701786</v>
       </c>
-      <c r="L49" s="6">
+      <c r="L49">
         <v>2</v>
       </c>
-      <c r="M49" s="12">
+      <c r="M49" s="10">
         <f t="shared" si="9"/>
         <v>9.7087378640776691E-3</v>
       </c>
-      <c r="N49" s="10">
+      <c r="N49" s="8">
         <v>0.29009397994530817</v>
       </c>
-      <c r="O49" s="6">
+      <c r="O49">
         <v>8</v>
       </c>
-      <c r="P49" s="12">
+      <c r="P49" s="10">
         <f t="shared" si="10"/>
         <v>3.8834951456310676E-2</v>
       </c>
-      <c r="T49" s="5">
+      <c r="T49" s="1">
         <v>-1.0692780198961159E-2</v>
       </c>
-      <c r="U49" s="6">
+      <c r="U49">
         <v>8</v>
       </c>
-      <c r="V49" s="12">
+      <c r="V49" s="10">
         <f t="shared" si="11"/>
         <v>3.8834951456310676E-2</v>
       </c>
-      <c r="W49" s="5">
+      <c r="W49" s="1">
         <v>-3.9964243721475707E-3</v>
       </c>
-      <c r="X49" s="6">
+      <c r="X49">
         <v>14</v>
       </c>
-      <c r="Y49" s="12">
+      <c r="Y49" s="10">
         <f t="shared" si="12"/>
         <v>6.8292682926829273E-2</v>
       </c>
-      <c r="AC49" s="5">
+      <c r="AC49" s="1">
         <v>2.7185095101106471</v>
       </c>
-      <c r="AD49" s="6">
-        <v>0</v>
-      </c>
-      <c r="AE49" s="12">
+      <c r="AD49">
+        <v>0</v>
+      </c>
+      <c r="AE49" s="10">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="AF49" s="5">
+      <c r="AF49" s="1">
         <v>2.2772298547355097</v>
       </c>
-      <c r="AG49" s="6">
+      <c r="AG49">
         <v>3</v>
       </c>
-      <c r="AH49" s="12">
+      <c r="AH49" s="10">
         <f t="shared" si="14"/>
         <v>1.4563106796116505E-2</v>
       </c>
@@ -13303,63 +13090,63 @@
       <c r="G50" s="2">
         <v>3.0825452292184101</v>
       </c>
-      <c r="K50" s="10">
+      <c r="K50" s="8">
         <v>0.45250172207229944</v>
       </c>
-      <c r="L50" s="6">
+      <c r="L50">
         <v>2</v>
       </c>
-      <c r="M50" s="12">
+      <c r="M50" s="10">
         <f t="shared" si="9"/>
         <v>9.7087378640776691E-3</v>
       </c>
-      <c r="N50" s="10">
+      <c r="N50" s="8">
         <v>0.3381826056069448</v>
       </c>
-      <c r="O50" s="6">
+      <c r="O50">
         <v>9</v>
       </c>
-      <c r="P50" s="12">
+      <c r="P50" s="10">
         <f t="shared" si="10"/>
         <v>4.3689320388349516E-2</v>
       </c>
-      <c r="T50" s="5">
+      <c r="T50" s="1">
         <v>-6.1646826286640907E-3</v>
       </c>
-      <c r="U50" s="6">
+      <c r="U50">
         <v>19</v>
       </c>
-      <c r="V50" s="12">
+      <c r="V50" s="10">
         <f t="shared" si="11"/>
         <v>9.2233009708737865E-2</v>
       </c>
-      <c r="W50" s="5">
+      <c r="W50" s="1">
         <v>6.5438478463017598E-4</v>
       </c>
-      <c r="X50" s="6">
+      <c r="X50">
         <v>25</v>
       </c>
-      <c r="Y50" s="12">
+      <c r="Y50" s="10">
         <f t="shared" si="12"/>
         <v>0.12195121951219512</v>
       </c>
-      <c r="AC50" s="5">
+      <c r="AC50" s="1">
         <v>2.7699835622143265</v>
       </c>
-      <c r="AD50" s="6">
+      <c r="AD50">
         <v>2</v>
       </c>
-      <c r="AE50" s="12">
+      <c r="AE50" s="10">
         <f t="shared" si="13"/>
         <v>9.7560975609756097E-3</v>
       </c>
-      <c r="AF50" s="5">
+      <c r="AF50" s="1">
         <v>2.3731570884216677</v>
       </c>
-      <c r="AG50" s="6">
+      <c r="AG50">
         <v>4</v>
       </c>
-      <c r="AH50" s="12">
+      <c r="AH50" s="10">
         <f t="shared" si="14"/>
         <v>1.9417475728155338E-2</v>
       </c>
@@ -13386,63 +13173,63 @@
       <c r="G51" s="2">
         <v>2.8873200961373899</v>
       </c>
-      <c r="K51" s="10">
+      <c r="K51" s="8">
         <v>0.49222011785758102</v>
       </c>
-      <c r="L51" s="6">
+      <c r="L51">
         <v>6</v>
       </c>
-      <c r="M51" s="12">
+      <c r="M51" s="10">
         <f t="shared" si="9"/>
         <v>2.9126213592233011E-2</v>
       </c>
-      <c r="N51" s="10">
+      <c r="N51" s="8">
         <v>0.38627123126858143</v>
       </c>
-      <c r="O51" s="6">
+      <c r="O51">
         <v>6</v>
       </c>
-      <c r="P51" s="12">
+      <c r="P51" s="10">
         <f t="shared" si="10"/>
         <v>2.9126213592233011E-2</v>
       </c>
-      <c r="T51" s="5">
+      <c r="T51" s="1">
         <v>-1.6365850583670224E-3</v>
       </c>
-      <c r="U51" s="6">
+      <c r="U51">
         <v>13</v>
       </c>
-      <c r="V51" s="12">
+      <c r="V51" s="10">
         <f t="shared" si="11"/>
         <v>6.3106796116504854E-2</v>
       </c>
-      <c r="W51" s="5">
+      <c r="W51" s="1">
         <v>5.3051939414079227E-3</v>
       </c>
-      <c r="X51" s="6">
+      <c r="X51">
         <v>28</v>
       </c>
-      <c r="Y51" s="12">
+      <c r="Y51" s="10">
         <f t="shared" si="12"/>
         <v>0.13658536585365855</v>
       </c>
-      <c r="AC51" s="5">
+      <c r="AC51" s="1">
         <v>2.8214576143180059</v>
       </c>
-      <c r="AD51" s="6">
+      <c r="AD51">
         <v>5</v>
       </c>
-      <c r="AE51" s="12">
+      <c r="AE51" s="10">
         <f t="shared" si="13"/>
         <v>2.4390243902439025E-2</v>
       </c>
-      <c r="AF51" s="5">
+      <c r="AF51" s="1">
         <v>2.4690843221078258</v>
       </c>
-      <c r="AG51" s="6">
+      <c r="AG51">
         <v>3</v>
       </c>
-      <c r="AH51" s="12">
+      <c r="AH51" s="10">
         <f t="shared" si="14"/>
         <v>1.4563106796116505E-2</v>
       </c>
@@ -13469,63 +13256,63 @@
       <c r="G52" s="2">
         <v>3.3649455208504699</v>
       </c>
-      <c r="K52" s="10">
+      <c r="K52" s="8">
         <v>0.5319385136428626</v>
       </c>
-      <c r="L52" s="6">
+      <c r="L52">
         <v>4</v>
       </c>
-      <c r="M52" s="12">
+      <c r="M52" s="10">
         <f t="shared" si="9"/>
         <v>1.9417475728155338E-2</v>
       </c>
-      <c r="N52" s="10">
+      <c r="N52" s="8">
         <v>0.43435985693021806</v>
       </c>
-      <c r="O52" s="6">
+      <c r="O52">
         <v>16</v>
       </c>
-      <c r="P52" s="12">
+      <c r="P52" s="10">
         <f t="shared" si="10"/>
         <v>7.7669902912621352E-2</v>
       </c>
-      <c r="T52" s="5">
+      <c r="T52" s="1">
         <v>2.8915125119300458E-3</v>
       </c>
-      <c r="U52" s="6">
+      <c r="U52">
         <v>22</v>
       </c>
-      <c r="V52" s="12">
+      <c r="V52" s="10">
         <f t="shared" si="11"/>
         <v>0.10679611650485436</v>
       </c>
-      <c r="W52" s="5">
+      <c r="W52" s="1">
         <v>9.9560030981856694E-3</v>
       </c>
-      <c r="X52" s="6">
+      <c r="X52">
         <v>31</v>
       </c>
-      <c r="Y52" s="12">
+      <c r="Y52" s="10">
         <f t="shared" si="12"/>
         <v>0.15121951219512195</v>
       </c>
-      <c r="AC52" s="5">
+      <c r="AC52" s="1">
         <v>2.8729316664216853</v>
       </c>
-      <c r="AD52" s="6">
+      <c r="AD52">
         <v>3</v>
       </c>
-      <c r="AE52" s="12">
+      <c r="AE52" s="10">
         <f t="shared" si="13"/>
         <v>1.4634146341463415E-2</v>
       </c>
-      <c r="AF52" s="5">
+      <c r="AF52" s="1">
         <v>2.5650115557939839</v>
       </c>
-      <c r="AG52" s="6">
+      <c r="AG52">
         <v>1</v>
       </c>
-      <c r="AH52" s="12">
+      <c r="AH52" s="10">
         <f t="shared" si="14"/>
         <v>4.8543689320388345E-3</v>
       </c>
@@ -13552,63 +13339,63 @@
       <c r="G53" s="2">
         <v>3.1995431843787601</v>
       </c>
-      <c r="K53" s="10">
+      <c r="K53" s="8">
         <v>0.57165690942814418</v>
       </c>
-      <c r="L53" s="6">
+      <c r="L53">
         <v>9</v>
       </c>
-      <c r="M53" s="12">
+      <c r="M53" s="10">
         <f t="shared" si="9"/>
         <v>4.3689320388349516E-2</v>
       </c>
-      <c r="N53" s="10">
+      <c r="N53" s="8">
         <v>0.48244848259185469</v>
       </c>
-      <c r="O53" s="6">
+      <c r="O53">
         <v>12</v>
       </c>
-      <c r="P53" s="12">
+      <c r="P53" s="10">
         <f t="shared" si="10"/>
         <v>5.8252427184466021E-2</v>
       </c>
-      <c r="T53" s="5">
+      <c r="T53" s="1">
         <v>7.4196100822271141E-3</v>
       </c>
-      <c r="U53" s="6">
+      <c r="U53">
         <v>33</v>
       </c>
-      <c r="V53" s="12">
+      <c r="V53" s="10">
         <f t="shared" si="11"/>
         <v>0.16019417475728157</v>
       </c>
-      <c r="W53" s="5">
+      <c r="W53" s="1">
         <v>1.4606812254963415E-2</v>
       </c>
-      <c r="X53" s="6">
+      <c r="X53">
         <v>42</v>
       </c>
-      <c r="Y53" s="12">
+      <c r="Y53" s="10">
         <f t="shared" si="12"/>
         <v>0.20487804878048779</v>
       </c>
-      <c r="AC53" s="5">
+      <c r="AC53" s="1">
         <v>2.9244057185253647</v>
       </c>
-      <c r="AD53" s="6">
+      <c r="AD53">
         <v>7</v>
       </c>
-      <c r="AE53" s="12">
+      <c r="AE53" s="10">
         <f t="shared" si="13"/>
         <v>3.4146341463414637E-2</v>
       </c>
-      <c r="AF53" s="5">
+      <c r="AF53" s="1">
         <v>2.660938789480142</v>
       </c>
-      <c r="AG53" s="6">
+      <c r="AG53">
         <v>11</v>
       </c>
-      <c r="AH53" s="12">
+      <c r="AH53" s="10">
         <f t="shared" si="14"/>
         <v>5.3398058252427182E-2</v>
       </c>
@@ -13635,63 +13422,63 @@
       <c r="G54" s="2">
         <v>3.2336083457401399</v>
       </c>
-      <c r="K54" s="10">
+      <c r="K54" s="8">
         <v>0.61137530521342576</v>
       </c>
-      <c r="L54" s="6">
+      <c r="L54">
         <v>12</v>
       </c>
-      <c r="M54" s="12">
+      <c r="M54" s="10">
         <f t="shared" si="9"/>
         <v>5.8252427184466021E-2</v>
       </c>
-      <c r="N54" s="10">
+      <c r="N54" s="8">
         <v>0.53053710825349132</v>
       </c>
-      <c r="O54" s="6">
+      <c r="O54">
         <v>31</v>
       </c>
-      <c r="P54" s="12">
+      <c r="P54" s="10">
         <f t="shared" si="10"/>
         <v>0.15048543689320387</v>
       </c>
-      <c r="T54" s="5">
+      <c r="T54" s="1">
         <v>1.1947707652524182E-2</v>
       </c>
-      <c r="U54" s="6">
+      <c r="U54">
         <v>23</v>
       </c>
-      <c r="V54" s="12">
+      <c r="V54" s="10">
         <f t="shared" si="11"/>
         <v>0.11165048543689321</v>
       </c>
-      <c r="W54" s="5">
+      <c r="W54" s="1">
         <v>1.9257621411741161E-2</v>
       </c>
-      <c r="X54" s="6">
+      <c r="X54">
         <v>17</v>
       </c>
-      <c r="Y54" s="12">
+      <c r="Y54" s="10">
         <f t="shared" si="12"/>
         <v>8.2926829268292687E-2</v>
       </c>
-      <c r="AC54" s="5">
+      <c r="AC54" s="1">
         <v>2.9758797706290441</v>
       </c>
-      <c r="AD54" s="6">
+      <c r="AD54">
         <v>29</v>
       </c>
-      <c r="AE54" s="12">
+      <c r="AE54" s="10">
         <f t="shared" si="13"/>
         <v>0.14146341463414633</v>
       </c>
-      <c r="AF54" s="5">
+      <c r="AF54" s="1">
         <v>2.7568660231663</v>
       </c>
-      <c r="AG54" s="6">
+      <c r="AG54">
         <v>14</v>
       </c>
-      <c r="AH54" s="12">
+      <c r="AH54" s="10">
         <f t="shared" si="14"/>
         <v>6.7961165048543687E-2</v>
       </c>
@@ -13718,63 +13505,63 @@
       <c r="G55" s="2">
         <v>2.9413315247701299</v>
       </c>
-      <c r="K55" s="10">
+      <c r="K55" s="8">
         <v>0.65109370099870734</v>
       </c>
-      <c r="L55" s="6">
+      <c r="L55">
         <v>14</v>
       </c>
-      <c r="M55" s="12">
+      <c r="M55" s="10">
         <f t="shared" si="9"/>
         <v>6.7961165048543687E-2</v>
       </c>
-      <c r="N55" s="10">
+      <c r="N55" s="8">
         <v>0.57862573391512795</v>
       </c>
-      <c r="O55" s="6">
+      <c r="O55">
         <v>14</v>
       </c>
-      <c r="P55" s="12">
+      <c r="P55" s="10">
         <f t="shared" si="10"/>
         <v>6.7961165048543687E-2</v>
       </c>
-      <c r="T55" s="5">
+      <c r="T55" s="1">
         <v>1.6475805222821251E-2</v>
       </c>
-      <c r="U55" s="6">
+      <c r="U55">
         <v>19</v>
       </c>
-      <c r="V55" s="12">
+      <c r="V55" s="10">
         <f t="shared" si="11"/>
         <v>9.2233009708737865E-2</v>
       </c>
-      <c r="W55" s="5">
+      <c r="W55" s="1">
         <v>2.3908430568518907E-2</v>
       </c>
-      <c r="X55" s="6">
+      <c r="X55">
         <v>8</v>
       </c>
-      <c r="Y55" s="12">
+      <c r="Y55" s="10">
         <f t="shared" si="12"/>
         <v>3.9024390243902439E-2</v>
       </c>
-      <c r="AC55" s="5">
+      <c r="AC55" s="1">
         <v>3.0273538227327235</v>
       </c>
-      <c r="AD55" s="6">
+      <c r="AD55">
         <v>14</v>
       </c>
-      <c r="AE55" s="12">
+      <c r="AE55" s="10">
         <f t="shared" si="13"/>
         <v>6.8292682926829273E-2</v>
       </c>
-      <c r="AF55" s="5">
+      <c r="AF55" s="1">
         <v>2.8527932568524581</v>
       </c>
-      <c r="AG55" s="6">
+      <c r="AG55">
         <v>14</v>
       </c>
-      <c r="AH55" s="12">
+      <c r="AH55" s="10">
         <f t="shared" si="14"/>
         <v>6.7961165048543687E-2</v>
       </c>
@@ -13801,63 +13588,63 @@
       <c r="G56" s="2">
         <v>1.8862259252790099</v>
       </c>
-      <c r="K56" s="10">
+      <c r="K56" s="8">
         <v>0.69081209678398892</v>
       </c>
-      <c r="L56" s="6">
+      <c r="L56">
         <v>20</v>
       </c>
-      <c r="M56" s="12">
+      <c r="M56" s="10">
         <f t="shared" si="9"/>
         <v>9.7087378640776698E-2</v>
       </c>
-      <c r="N56" s="10">
+      <c r="N56" s="8">
         <v>0.62671435957676458</v>
       </c>
-      <c r="O56" s="6">
+      <c r="O56">
         <v>25</v>
       </c>
-      <c r="P56" s="12">
+      <c r="P56" s="10">
         <f t="shared" si="10"/>
         <v>0.12135922330097088</v>
       </c>
-      <c r="T56" s="5">
+      <c r="T56" s="1">
         <v>2.1003902793118319E-2</v>
       </c>
-      <c r="U56" s="6">
+      <c r="U56">
         <v>21</v>
       </c>
-      <c r="V56" s="12">
+      <c r="V56" s="10">
         <f t="shared" si="11"/>
         <v>0.10194174757281553</v>
       </c>
-      <c r="W56" s="5">
+      <c r="W56" s="1">
         <v>2.8559239725296653E-2</v>
       </c>
-      <c r="X56" s="6">
+      <c r="X56">
         <v>7</v>
       </c>
-      <c r="Y56" s="12">
+      <c r="Y56" s="10">
         <f t="shared" si="12"/>
         <v>3.4146341463414637E-2</v>
       </c>
-      <c r="AC56" s="5">
+      <c r="AC56" s="1">
         <v>3.0788278748364029</v>
       </c>
-      <c r="AD56" s="6">
+      <c r="AD56">
         <v>19</v>
       </c>
-      <c r="AE56" s="12">
+      <c r="AE56" s="10">
         <f t="shared" si="13"/>
         <v>9.2682926829268292E-2</v>
       </c>
-      <c r="AF56" s="5">
+      <c r="AF56" s="1">
         <v>2.9487204905386162</v>
       </c>
-      <c r="AG56" s="6">
+      <c r="AG56">
         <v>28</v>
       </c>
-      <c r="AH56" s="12">
+      <c r="AH56" s="10">
         <f t="shared" si="14"/>
         <v>0.13592233009708737</v>
       </c>
@@ -13884,63 +13671,63 @@
       <c r="G57" s="2">
         <v>2.8422128301349301</v>
       </c>
-      <c r="K57" s="10">
+      <c r="K57" s="8">
         <v>0.7305304925692705</v>
       </c>
-      <c r="L57" s="6">
+      <c r="L57">
         <v>14</v>
       </c>
-      <c r="M57" s="12">
+      <c r="M57" s="10">
         <f t="shared" si="9"/>
         <v>6.7961165048543687E-2</v>
       </c>
-      <c r="N57" s="10">
+      <c r="N57" s="8">
         <v>0.67480298523840121</v>
       </c>
-      <c r="O57" s="6">
+      <c r="O57">
         <v>9</v>
       </c>
-      <c r="P57" s="12">
+      <c r="P57" s="10">
         <f t="shared" si="10"/>
         <v>4.3689320388349516E-2</v>
       </c>
-      <c r="T57" s="5">
+      <c r="T57" s="1">
         <v>2.5532000363415387E-2</v>
       </c>
-      <c r="U57" s="6">
+      <c r="U57">
         <v>17</v>
       </c>
-      <c r="V57" s="12">
+      <c r="V57" s="10">
         <f t="shared" si="11"/>
         <v>8.2524271844660199E-2</v>
       </c>
-      <c r="W57" s="5">
+      <c r="W57" s="1">
         <v>3.3210048882074399E-2</v>
       </c>
-      <c r="X57" s="6">
+      <c r="X57">
         <v>8</v>
       </c>
-      <c r="Y57" s="12">
+      <c r="Y57" s="10">
         <f t="shared" si="12"/>
         <v>3.9024390243902439E-2</v>
       </c>
-      <c r="AC57" s="5">
+      <c r="AC57" s="1">
         <v>3.1303019269400822</v>
       </c>
-      <c r="AD57" s="6">
+      <c r="AD57">
         <v>23</v>
       </c>
-      <c r="AE57" s="12">
+      <c r="AE57" s="10">
         <f t="shared" si="13"/>
         <v>0.11219512195121951</v>
       </c>
-      <c r="AF57" s="5">
+      <c r="AF57" s="1">
         <v>3.0446477242247743</v>
       </c>
-      <c r="AG57" s="6">
+      <c r="AG57">
         <v>23</v>
       </c>
-      <c r="AH57" s="12">
+      <c r="AH57" s="10">
         <f t="shared" si="14"/>
         <v>0.11165048543689321</v>
       </c>
@@ -13967,63 +13754,63 @@
       <c r="G58" s="2">
         <v>2.61292294689436</v>
       </c>
-      <c r="K58" s="10">
+      <c r="K58" s="8">
         <v>0.77024888835455207</v>
       </c>
-      <c r="L58" s="6">
+      <c r="L58">
         <v>29</v>
       </c>
-      <c r="M58" s="12">
+      <c r="M58" s="10">
         <f t="shared" si="9"/>
         <v>0.14077669902912621</v>
       </c>
-      <c r="N58" s="10">
+      <c r="N58" s="8">
         <v>0.72289161090003784</v>
       </c>
-      <c r="O58" s="6">
+      <c r="O58">
         <v>12</v>
       </c>
-      <c r="P58" s="12">
+      <c r="P58" s="10">
         <f t="shared" si="10"/>
         <v>5.8252427184466021E-2</v>
       </c>
-      <c r="T58" s="5">
+      <c r="T58" s="1">
         <v>3.0060097933712455E-2</v>
       </c>
-      <c r="U58" s="6">
+      <c r="U58">
         <v>6</v>
       </c>
-      <c r="V58" s="12">
+      <c r="V58" s="10">
         <f t="shared" si="11"/>
         <v>2.9126213592233011E-2</v>
       </c>
-      <c r="W58" s="5">
+      <c r="W58" s="1">
         <v>3.7860858038852148E-2</v>
       </c>
-      <c r="X58" s="6">
+      <c r="X58">
         <v>2</v>
       </c>
-      <c r="Y58" s="12">
+      <c r="Y58" s="10">
         <f t="shared" si="12"/>
         <v>9.7560975609756097E-3</v>
       </c>
-      <c r="AC58" s="5">
+      <c r="AC58" s="1">
         <v>3.1817759790437616</v>
       </c>
-      <c r="AD58" s="6">
+      <c r="AD58">
         <v>28</v>
       </c>
-      <c r="AE58" s="12">
+      <c r="AE58" s="10">
         <f t="shared" si="13"/>
         <v>0.13658536585365855</v>
       </c>
-      <c r="AF58" s="5">
+      <c r="AF58" s="1">
         <v>3.1405749579109323</v>
       </c>
-      <c r="AG58" s="6">
+      <c r="AG58">
         <v>25</v>
       </c>
-      <c r="AH58" s="12">
+      <c r="AH58" s="10">
         <f t="shared" si="14"/>
         <v>0.12135922330097088</v>
       </c>
@@ -14050,63 +13837,63 @@
       <c r="G59" s="2">
         <v>3.1838281484811901</v>
       </c>
-      <c r="K59" s="10">
+      <c r="K59" s="8">
         <v>0.80996728413983365</v>
       </c>
-      <c r="L59" s="6">
+      <c r="L59">
         <v>29</v>
       </c>
-      <c r="M59" s="12">
+      <c r="M59" s="10">
         <f t="shared" si="9"/>
         <v>0.14077669902912621</v>
       </c>
-      <c r="N59" s="10">
+      <c r="N59" s="8">
         <v>0.77098023656167447</v>
       </c>
-      <c r="O59" s="6">
+      <c r="O59">
         <v>5</v>
       </c>
-      <c r="P59" s="12">
+      <c r="P59" s="10">
         <f t="shared" si="10"/>
         <v>2.4271844660194174E-2</v>
       </c>
-      <c r="T59" s="5">
+      <c r="T59" s="1">
         <v>3.4588195504009524E-2</v>
       </c>
-      <c r="U59" s="6">
+      <c r="U59">
         <v>10</v>
       </c>
-      <c r="V59" s="12">
+      <c r="V59" s="10">
         <f t="shared" si="11"/>
         <v>4.8543689320388349E-2</v>
       </c>
-      <c r="W59" s="5">
+      <c r="W59" s="1">
         <v>4.2511667195629897E-2</v>
       </c>
-      <c r="X59" s="6">
+      <c r="X59">
         <v>1</v>
       </c>
-      <c r="Y59" s="12">
+      <c r="Y59" s="10">
         <f t="shared" si="12"/>
         <v>4.8780487804878049E-3</v>
       </c>
-      <c r="AC59" s="5">
+      <c r="AC59" s="1">
         <v>3.233250031147441</v>
       </c>
-      <c r="AD59" s="6">
+      <c r="AD59">
         <v>27</v>
       </c>
-      <c r="AE59" s="12">
+      <c r="AE59" s="10">
         <f t="shared" si="13"/>
         <v>0.13170731707317074</v>
       </c>
-      <c r="AF59" s="5">
+      <c r="AF59" s="1">
         <v>3.2365021915970904</v>
       </c>
-      <c r="AG59" s="6">
+      <c r="AG59">
         <v>34</v>
       </c>
-      <c r="AH59" s="12">
+      <c r="AH59" s="10">
         <f t="shared" si="14"/>
         <v>0.1650485436893204</v>
       </c>
@@ -14133,63 +13920,63 @@
       <c r="G60" s="2">
         <v>2.6479643847373899</v>
       </c>
-      <c r="K60" s="10">
+      <c r="K60" s="8">
         <v>0.84968567992511523</v>
       </c>
-      <c r="L60" s="6">
+      <c r="L60">
         <v>32</v>
       </c>
-      <c r="M60" s="12">
+      <c r="M60" s="10">
         <f t="shared" si="9"/>
         <v>0.1553398058252427</v>
       </c>
-      <c r="N60" s="10">
+      <c r="N60" s="8">
         <v>0.8190688622233111</v>
       </c>
-      <c r="O60" s="6">
+      <c r="O60">
         <v>6</v>
       </c>
-      <c r="P60" s="12">
+      <c r="P60" s="10">
         <f t="shared" si="10"/>
         <v>2.9126213592233011E-2</v>
       </c>
-      <c r="T60" s="5">
+      <c r="T60" s="1">
         <v>3.9116293074306592E-2</v>
       </c>
-      <c r="U60" s="6">
+      <c r="U60">
         <v>2</v>
       </c>
-      <c r="V60" s="12">
+      <c r="V60" s="10">
         <f t="shared" si="11"/>
         <v>9.7087378640776691E-3</v>
       </c>
-      <c r="W60" s="5">
+      <c r="W60" s="1">
         <v>4.7162476352407647E-2</v>
       </c>
-      <c r="X60" s="6">
-        <v>0</v>
-      </c>
-      <c r="Y60" s="12">
+      <c r="X60">
+        <v>0</v>
+      </c>
+      <c r="Y60" s="10">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="AC60" s="5">
+      <c r="AC60" s="1">
         <v>3.2847240832511204</v>
       </c>
-      <c r="AD60" s="6">
+      <c r="AD60">
         <v>31</v>
       </c>
-      <c r="AE60" s="12">
+      <c r="AE60" s="10">
         <f t="shared" si="13"/>
         <v>0.15121951219512195</v>
       </c>
-      <c r="AF60" s="5">
+      <c r="AF60" s="1">
         <v>3.3324294252832485</v>
       </c>
-      <c r="AG60" s="6">
+      <c r="AG60">
         <v>19</v>
       </c>
-      <c r="AH60" s="12">
+      <c r="AH60" s="10">
         <f t="shared" si="14"/>
         <v>9.2233009708737865E-2</v>
       </c>
@@ -14216,63 +14003,63 @@
       <c r="G61" s="2">
         <v>2.8582859427606202</v>
       </c>
-      <c r="K61" s="10">
+      <c r="K61" s="8">
         <v>0.88940407571039681</v>
       </c>
-      <c r="L61" s="6">
+      <c r="L61">
         <v>13</v>
       </c>
-      <c r="M61" s="12">
+      <c r="M61" s="10">
         <f t="shared" si="9"/>
         <v>6.3106796116504854E-2</v>
       </c>
-      <c r="N61" s="10">
+      <c r="N61" s="8">
         <v>0.86715748788494773</v>
       </c>
-      <c r="O61" s="6">
+      <c r="O61">
         <v>8</v>
       </c>
-      <c r="P61" s="12">
+      <c r="P61" s="10">
         <f t="shared" si="10"/>
         <v>3.8834951456310676E-2</v>
       </c>
-      <c r="T61" s="5">
+      <c r="T61" s="1">
         <v>4.364439064460366E-2</v>
       </c>
-      <c r="U61" s="6">
+      <c r="U61">
         <v>2</v>
       </c>
-      <c r="V61" s="12">
+      <c r="V61" s="10">
         <f t="shared" si="11"/>
         <v>9.7087378640776691E-3</v>
       </c>
-      <c r="W61" s="5">
+      <c r="W61" s="1">
         <v>5.1813285509185396E-2</v>
       </c>
-      <c r="X61" s="6">
-        <v>0</v>
-      </c>
-      <c r="Y61" s="12">
+      <c r="X61">
+        <v>0</v>
+      </c>
+      <c r="Y61" s="10">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="AC61" s="5">
+      <c r="AC61" s="1">
         <v>3.3361981353547998</v>
       </c>
-      <c r="AD61" s="6">
+      <c r="AD61">
         <v>9</v>
       </c>
-      <c r="AE61" s="12">
+      <c r="AE61" s="10">
         <f t="shared" si="13"/>
         <v>4.3902439024390241E-2</v>
       </c>
-      <c r="AF61" s="5">
+      <c r="AF61" s="1">
         <v>3.4283566589694066</v>
       </c>
-      <c r="AG61" s="6">
+      <c r="AG61">
         <v>5</v>
       </c>
-      <c r="AH61" s="12">
+      <c r="AH61" s="10">
         <f t="shared" si="14"/>
         <v>2.4271844660194174E-2</v>
       </c>
@@ -14299,63 +14086,63 @@
       <c r="G62" s="2">
         <v>2.8751345119722398</v>
       </c>
-      <c r="K62" s="10">
+      <c r="K62" s="8">
         <v>0.92912247149567839</v>
       </c>
-      <c r="L62" s="6">
+      <c r="L62">
         <v>9</v>
       </c>
-      <c r="M62" s="12">
+      <c r="M62" s="10">
         <f t="shared" si="9"/>
         <v>4.3689320388349516E-2</v>
       </c>
-      <c r="N62" s="10">
+      <c r="N62" s="8">
         <v>0.91524611354658436</v>
       </c>
-      <c r="O62" s="6">
+      <c r="O62">
         <v>1</v>
       </c>
-      <c r="P62" s="12">
+      <c r="P62" s="10">
         <f t="shared" si="10"/>
         <v>4.8543689320388345E-3</v>
       </c>
-      <c r="T62" s="5">
+      <c r="T62" s="1">
         <v>4.8172488214900729E-2</v>
       </c>
-      <c r="U62" s="6">
-        <v>0</v>
-      </c>
-      <c r="V62" s="12">
+      <c r="U62">
+        <v>0</v>
+      </c>
+      <c r="V62" s="10">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
-      <c r="W62" s="5">
+      <c r="W62" s="1">
         <v>5.6464094665963145E-2</v>
       </c>
-      <c r="X62" s="6">
-        <v>0</v>
-      </c>
-      <c r="Y62" s="12">
+      <c r="X62">
+        <v>0</v>
+      </c>
+      <c r="Y62" s="10">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="AC62" s="5">
+      <c r="AC62" s="1">
         <v>3.3876721874584792</v>
       </c>
-      <c r="AD62" s="6">
+      <c r="AD62">
         <v>6</v>
       </c>
-      <c r="AE62" s="12">
+      <c r="AE62" s="10">
         <f t="shared" si="13"/>
         <v>2.9268292682926831E-2</v>
       </c>
-      <c r="AF62" s="5">
+      <c r="AF62" s="1">
         <v>3.5242838926555646</v>
       </c>
-      <c r="AG62" s="6">
+      <c r="AG62">
         <v>1</v>
       </c>
-      <c r="AH62" s="12">
+      <c r="AH62" s="10">
         <f t="shared" si="14"/>
         <v>4.8543689320388345E-3</v>
       </c>
@@ -14382,63 +14169,63 @@
       <c r="G63" s="2">
         <v>2.7813876007042002</v>
       </c>
-      <c r="K63" s="10">
+      <c r="K63" s="8">
         <v>0.96884086728095997</v>
       </c>
-      <c r="L63" s="6">
+      <c r="L63">
         <v>7</v>
       </c>
-      <c r="M63" s="12">
+      <c r="M63" s="10">
         <f t="shared" si="9"/>
         <v>3.3980582524271843E-2</v>
       </c>
-      <c r="N63" s="10">
+      <c r="N63" s="8">
         <v>0.96333473920822099</v>
       </c>
-      <c r="O63" s="6">
+      <c r="O63">
         <v>2</v>
       </c>
-      <c r="P63" s="12">
+      <c r="P63" s="10">
         <f t="shared" si="10"/>
         <v>9.7087378640776691E-3</v>
       </c>
-      <c r="T63" s="5">
+      <c r="T63" s="1">
         <v>5.2700585785197797E-2</v>
       </c>
-      <c r="U63" s="6">
+      <c r="U63">
         <v>1</v>
       </c>
-      <c r="V63" s="12">
+      <c r="V63" s="10">
         <f t="shared" si="11"/>
         <v>4.8543689320388345E-3</v>
       </c>
-      <c r="W63" s="5">
+      <c r="W63" s="1">
         <v>6.1114903822740894E-2</v>
       </c>
-      <c r="X63" s="6">
-        <v>0</v>
-      </c>
-      <c r="Y63" s="12">
+      <c r="X63">
+        <v>0</v>
+      </c>
+      <c r="Y63" s="10">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="AC63" s="5">
+      <c r="AC63" s="1">
         <v>3.4391462395621586</v>
       </c>
-      <c r="AD63" s="6">
-        <v>0</v>
-      </c>
-      <c r="AE63" s="12">
+      <c r="AD63">
+        <v>0</v>
+      </c>
+      <c r="AE63" s="10">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="AF63" s="5">
+      <c r="AF63" s="1">
         <v>3.6202111263417227</v>
       </c>
-      <c r="AG63" s="6">
+      <c r="AG63">
         <v>1</v>
       </c>
-      <c r="AH63" s="12">
+      <c r="AH63" s="10">
         <f t="shared" si="14"/>
         <v>4.8543689320388345E-3</v>
       </c>
@@ -14465,40 +14252,40 @@
       <c r="G64" s="2">
         <v>3.2959015619510699</v>
       </c>
-      <c r="K64" s="7" t="s">
+      <c r="K64" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="L64" s="7">
-        <v>0</v>
-      </c>
-      <c r="N64" s="7" t="s">
+      <c r="L64" s="5">
+        <v>0</v>
+      </c>
+      <c r="N64" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="O64" s="7">
-        <v>0</v>
-      </c>
-      <c r="T64" s="7" t="s">
+      <c r="O64" s="5">
+        <v>0</v>
+      </c>
+      <c r="T64" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="U64" s="7">
-        <v>0</v>
-      </c>
-      <c r="W64" s="7" t="s">
+      <c r="U64" s="5">
+        <v>0</v>
+      </c>
+      <c r="W64" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="X64" s="7">
+      <c r="X64" s="5">
         <v>1</v>
       </c>
-      <c r="AC64" s="7" t="s">
+      <c r="AC64" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="AD64" s="7">
+      <c r="AD64" s="5">
         <v>1</v>
       </c>
-      <c r="AF64" s="7" t="s">
+      <c r="AF64" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="AG64" s="7">
+      <c r="AG64" s="5">
         <v>0</v>
       </c>
     </row>
@@ -14689,10 +14476,10 @@
       <c r="J71" t="s">
         <v>21</v>
       </c>
-      <c r="K71" s="11">
+      <c r="K71" s="9">
         <v>0.21419134736060999</v>
       </c>
-      <c r="L71" s="11">
+      <c r="L71" s="9">
         <v>4.8543689320388345E-3</v>
       </c>
     </row>
@@ -14721,10 +14508,10 @@
       <c r="J72" t="s">
         <v>21</v>
       </c>
-      <c r="K72" s="11">
+      <c r="K72" s="9">
         <v>0.25390974314589154</v>
       </c>
-      <c r="L72" s="11">
+      <c r="L72" s="9">
         <v>4.8543689320388345E-3</v>
       </c>
     </row>
@@ -14753,10 +14540,10 @@
       <c r="J73" t="s">
         <v>21</v>
       </c>
-      <c r="K73" s="11">
+      <c r="K73" s="9">
         <v>0.29362813893117312</v>
       </c>
-      <c r="L73" s="11">
+      <c r="L73" s="9">
         <v>4.8543689320388345E-3</v>
       </c>
       <c r="T73" t="s">
@@ -14803,10 +14590,10 @@
       <c r="J74" t="s">
         <v>21</v>
       </c>
-      <c r="K74" s="11">
+      <c r="K74" s="9">
         <v>0.3333465347164547</v>
       </c>
-      <c r="L74" s="11">
+      <c r="L74" s="9">
         <v>4.8543689320388345E-3</v>
       </c>
       <c r="T74" t="s">
@@ -14853,10 +14640,10 @@
       <c r="J75" t="s">
         <v>21</v>
       </c>
-      <c r="K75" s="11">
+      <c r="K75" s="9">
         <v>0.37306493050173628</v>
       </c>
-      <c r="L75" s="11">
+      <c r="L75" s="9">
         <v>0</v>
       </c>
       <c r="T75" t="s">
@@ -14903,10 +14690,10 @@
       <c r="J76" t="s">
         <v>21</v>
       </c>
-      <c r="K76" s="11">
+      <c r="K76" s="9">
         <v>0.41278332628701786</v>
       </c>
-      <c r="L76" s="11">
+      <c r="L76" s="9">
         <v>9.7087378640776691E-3</v>
       </c>
       <c r="T76" t="s">
@@ -14953,10 +14740,10 @@
       <c r="J77" t="s">
         <v>21</v>
       </c>
-      <c r="K77" s="11">
+      <c r="K77" s="9">
         <v>0.45250172207229944</v>
       </c>
-      <c r="L77" s="11">
+      <c r="L77" s="9">
         <v>9.7087378640776691E-3</v>
       </c>
       <c r="T77" t="s">
@@ -15003,10 +14790,10 @@
       <c r="J78" t="s">
         <v>21</v>
       </c>
-      <c r="K78" s="11">
+      <c r="K78" s="9">
         <v>0.49222011785758102</v>
       </c>
-      <c r="L78" s="11">
+      <c r="L78" s="9">
         <v>2.9126213592233011E-2</v>
       </c>
       <c r="T78" t="s">
@@ -15053,10 +14840,10 @@
       <c r="J79" t="s">
         <v>21</v>
       </c>
-      <c r="K79" s="11">
+      <c r="K79" s="9">
         <v>0.5319385136428626</v>
       </c>
-      <c r="L79" s="11">
+      <c r="L79" s="9">
         <v>1.9417475728155338E-2</v>
       </c>
       <c r="T79" t="s">
@@ -15103,10 +14890,10 @@
       <c r="J80" t="s">
         <v>21</v>
       </c>
-      <c r="K80" s="11">
+      <c r="K80" s="9">
         <v>0.57165690942814418</v>
       </c>
-      <c r="L80" s="11">
+      <c r="L80" s="9">
         <v>4.3689320388349516E-2</v>
       </c>
       <c r="T80" t="s">
@@ -15153,10 +14940,10 @@
       <c r="J81" t="s">
         <v>21</v>
       </c>
-      <c r="K81" s="11">
+      <c r="K81" s="9">
         <v>0.61137530521342576</v>
       </c>
-      <c r="L81" s="11">
+      <c r="L81" s="9">
         <v>5.8252427184466021E-2</v>
       </c>
       <c r="T81" t="s">
@@ -15203,10 +14990,10 @@
       <c r="J82" t="s">
         <v>21</v>
       </c>
-      <c r="K82" s="11">
+      <c r="K82" s="9">
         <v>0.65109370099870734</v>
       </c>
-      <c r="L82" s="11">
+      <c r="L82" s="9">
         <v>6.7961165048543687E-2</v>
       </c>
       <c r="T82" t="s">
@@ -15253,10 +15040,10 @@
       <c r="J83" t="s">
         <v>21</v>
       </c>
-      <c r="K83" s="11">
+      <c r="K83" s="9">
         <v>0.69081209678398892</v>
       </c>
-      <c r="L83" s="11">
+      <c r="L83" s="9">
         <v>9.7087378640776698E-2</v>
       </c>
       <c r="T83" t="s">
@@ -15303,10 +15090,10 @@
       <c r="J84" t="s">
         <v>21</v>
       </c>
-      <c r="K84" s="11">
+      <c r="K84" s="9">
         <v>0.7305304925692705</v>
       </c>
-      <c r="L84" s="11">
+      <c r="L84" s="9">
         <v>6.7961165048543687E-2</v>
       </c>
       <c r="T84" t="s">
@@ -15353,10 +15140,10 @@
       <c r="J85" t="s">
         <v>21</v>
       </c>
-      <c r="K85" s="11">
+      <c r="K85" s="9">
         <v>0.77024888835455207</v>
       </c>
-      <c r="L85" s="11">
+      <c r="L85" s="9">
         <v>0.14077669902912621</v>
       </c>
       <c r="T85" t="s">
@@ -15403,10 +15190,10 @@
       <c r="J86" t="s">
         <v>21</v>
       </c>
-      <c r="K86" s="11">
+      <c r="K86" s="9">
         <v>0.80996728413983365</v>
       </c>
-      <c r="L86" s="11">
+      <c r="L86" s="9">
         <v>0.14077669902912621</v>
       </c>
       <c r="T86" t="s">
@@ -15453,10 +15240,10 @@
       <c r="J87" t="s">
         <v>21</v>
       </c>
-      <c r="K87" s="11">
+      <c r="K87" s="9">
         <v>0.84968567992511523</v>
       </c>
-      <c r="L87" s="11">
+      <c r="L87" s="9">
         <v>0.1553398058252427</v>
       </c>
       <c r="T87" t="s">
@@ -15503,10 +15290,10 @@
       <c r="J88" t="s">
         <v>21</v>
       </c>
-      <c r="K88" s="11">
+      <c r="K88" s="9">
         <v>0.88940407571039681</v>
       </c>
-      <c r="L88" s="11">
+      <c r="L88" s="9">
         <v>6.3106796116504854E-2</v>
       </c>
       <c r="T88" t="s">
@@ -15553,10 +15340,10 @@
       <c r="J89" t="s">
         <v>21</v>
       </c>
-      <c r="K89" s="11">
+      <c r="K89" s="9">
         <v>0.92912247149567839</v>
       </c>
-      <c r="L89" s="11">
+      <c r="L89" s="9">
         <v>4.3689320388349516E-2</v>
       </c>
       <c r="T89" t="s">
@@ -15603,10 +15390,10 @@
       <c r="J90" t="s">
         <v>21</v>
       </c>
-      <c r="K90" s="11">
+      <c r="K90" s="9">
         <v>0.96884086728095997</v>
       </c>
-      <c r="L90" s="11">
+      <c r="L90" s="9">
         <v>3.3980582524271843E-2</v>
       </c>
       <c r="T90" t="s">
@@ -15653,10 +15440,10 @@
       <c r="J91" t="s">
         <v>22</v>
       </c>
-      <c r="K91" s="9">
+      <c r="K91" s="7">
         <v>4.9650851637125001E-2</v>
       </c>
-      <c r="L91" s="11">
+      <c r="L91" s="9">
         <v>4.8543689320388345E-3</v>
       </c>
       <c r="T91" t="s">
@@ -15703,10 +15490,10 @@
       <c r="J92" t="s">
         <v>22</v>
       </c>
-      <c r="K92" s="9">
+      <c r="K92" s="7">
         <v>9.7739477298761632E-2</v>
       </c>
-      <c r="L92" s="11">
+      <c r="L92" s="9">
         <v>0.10194174757281553</v>
       </c>
       <c r="T92" t="s">
@@ -15753,10 +15540,10 @@
       <c r="J93" t="s">
         <v>22</v>
       </c>
-      <c r="K93" s="9">
+      <c r="K93" s="7">
         <v>0.14582810296039828</v>
       </c>
-      <c r="L93" s="11">
+      <c r="L93" s="9">
         <v>1.9417475728155338E-2</v>
       </c>
       <c r="T93" t="s">
@@ -15803,10 +15590,10 @@
       <c r="J94" t="s">
         <v>22</v>
       </c>
-      <c r="K94" s="9">
+      <c r="K94" s="7">
         <v>0.19391672862203491</v>
       </c>
-      <c r="L94" s="11">
+      <c r="L94" s="9">
         <v>4.8543689320388349E-2</v>
       </c>
       <c r="T94" t="s">
@@ -15853,10 +15640,10 @@
       <c r="J95" t="s">
         <v>22</v>
       </c>
-      <c r="K95" s="9">
+      <c r="K95" s="7">
         <v>0.24200535428367154</v>
       </c>
-      <c r="L95" s="11">
+      <c r="L95" s="9">
         <v>2.9126213592233011E-2</v>
       </c>
       <c r="T95" t="s">
@@ -15903,10 +15690,10 @@
       <c r="J96" t="s">
         <v>22</v>
       </c>
-      <c r="K96" s="9">
+      <c r="K96" s="7">
         <v>0.29009397994530817</v>
       </c>
-      <c r="L96" s="11">
+      <c r="L96" s="9">
         <v>3.8834951456310676E-2</v>
       </c>
       <c r="T96" t="s">
@@ -15953,10 +15740,10 @@
       <c r="J97" t="s">
         <v>22</v>
       </c>
-      <c r="K97" s="9">
+      <c r="K97" s="7">
         <v>0.3381826056069448</v>
       </c>
-      <c r="L97" s="11">
+      <c r="L97" s="9">
         <v>4.3689320388349516E-2</v>
       </c>
       <c r="T97" t="s">
@@ -16003,10 +15790,10 @@
       <c r="J98" t="s">
         <v>22</v>
       </c>
-      <c r="K98" s="9">
+      <c r="K98" s="7">
         <v>0.38627123126858143</v>
       </c>
-      <c r="L98" s="11">
+      <c r="L98" s="9">
         <v>2.9126213592233011E-2</v>
       </c>
       <c r="T98" t="s">
@@ -16053,10 +15840,10 @@
       <c r="J99" t="s">
         <v>22</v>
       </c>
-      <c r="K99" s="9">
+      <c r="K99" s="7">
         <v>0.43435985693021806</v>
       </c>
-      <c r="L99" s="11">
+      <c r="L99" s="9">
         <v>7.7669902912621352E-2</v>
       </c>
       <c r="T99" t="s">
@@ -16103,10 +15890,10 @@
       <c r="J100" t="s">
         <v>22</v>
       </c>
-      <c r="K100" s="9">
+      <c r="K100" s="7">
         <v>0.48244848259185469</v>
       </c>
-      <c r="L100" s="11">
+      <c r="L100" s="9">
         <v>5.8252427184466021E-2</v>
       </c>
       <c r="T100" t="s">
@@ -16153,10 +15940,10 @@
       <c r="J101" t="s">
         <v>22</v>
       </c>
-      <c r="K101" s="9">
+      <c r="K101" s="7">
         <v>0.53053710825349132</v>
       </c>
-      <c r="L101" s="11">
+      <c r="L101" s="9">
         <v>0.15048543689320387</v>
       </c>
       <c r="T101" t="s">
@@ -16203,10 +15990,10 @@
       <c r="J102" t="s">
         <v>22</v>
       </c>
-      <c r="K102" s="9">
+      <c r="K102" s="7">
         <v>0.57862573391512795</v>
       </c>
-      <c r="L102" s="11">
+      <c r="L102" s="9">
         <v>6.7961165048543687E-2</v>
       </c>
       <c r="T102" t="s">
@@ -16253,10 +16040,10 @@
       <c r="J103" t="s">
         <v>22</v>
       </c>
-      <c r="K103" s="9">
+      <c r="K103" s="7">
         <v>0.62671435957676458</v>
       </c>
-      <c r="L103" s="11">
+      <c r="L103" s="9">
         <v>0.12135922330097088</v>
       </c>
       <c r="T103" t="s">
@@ -16303,10 +16090,10 @@
       <c r="J104" t="s">
         <v>22</v>
       </c>
-      <c r="K104" s="9">
+      <c r="K104" s="7">
         <v>0.67480298523840121</v>
       </c>
-      <c r="L104" s="11">
+      <c r="L104" s="9">
         <v>4.3689320388349516E-2</v>
       </c>
       <c r="T104" t="s">
@@ -16353,10 +16140,10 @@
       <c r="J105" t="s">
         <v>22</v>
       </c>
-      <c r="K105" s="9">
+      <c r="K105" s="7">
         <v>0.72289161090003784</v>
       </c>
-      <c r="L105" s="11">
+      <c r="L105" s="9">
         <v>5.8252427184466021E-2</v>
       </c>
       <c r="T105" t="s">
@@ -16403,10 +16190,10 @@
       <c r="J106" t="s">
         <v>22</v>
       </c>
-      <c r="K106" s="9">
+      <c r="K106" s="7">
         <v>0.77098023656167447</v>
       </c>
-      <c r="L106" s="11">
+      <c r="L106" s="9">
         <v>2.4271844660194174E-2</v>
       </c>
       <c r="T106" t="s">
@@ -16453,10 +16240,10 @@
       <c r="J107" t="s">
         <v>22</v>
       </c>
-      <c r="K107" s="9">
+      <c r="K107" s="7">
         <v>0.8190688622233111</v>
       </c>
-      <c r="L107" s="11">
+      <c r="L107" s="9">
         <v>2.9126213592233011E-2</v>
       </c>
       <c r="T107" t="s">
@@ -16503,10 +16290,10 @@
       <c r="J108" t="s">
         <v>22</v>
       </c>
-      <c r="K108" s="9">
+      <c r="K108" s="7">
         <v>0.86715748788494773</v>
       </c>
-      <c r="L108" s="11">
+      <c r="L108" s="9">
         <v>3.8834951456310676E-2</v>
       </c>
       <c r="T108" t="s">
@@ -16553,10 +16340,10 @@
       <c r="J109" t="s">
         <v>22</v>
       </c>
-      <c r="K109" s="9">
+      <c r="K109" s="7">
         <v>0.91524611354658436</v>
       </c>
-      <c r="L109" s="11">
+      <c r="L109" s="9">
         <v>4.8543689320388345E-3</v>
       </c>
       <c r="T109" t="s">
@@ -16603,10 +16390,10 @@
       <c r="J110" t="s">
         <v>22</v>
       </c>
-      <c r="K110" s="9">
+      <c r="K110" s="7">
         <v>0.96333473920822099</v>
       </c>
-      <c r="L110" s="11">
+      <c r="L110" s="9">
         <v>9.7087378640776691E-3</v>
       </c>
       <c r="T110" t="s">

</xml_diff>